<commit_message>
Build Cham Cong robot implementation with Excel data processing
</commit_message>
<xml_diff>
--- a/Library/Data/Input/Tạo dữ liệu tính lương.xlsx
+++ b/Library/Data/Input/Tạo dữ liệu tính lương.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29704"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HoangTT\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huyhh1\workspace\kofax\cham-cong\Library\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{34B831DE-268F-417B-8CC5-72818CC02A58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8161C76B-DD29-4A17-8BC7-BEA913895D2B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B3A814C-F636-4F83-B75C-DDC998CF87D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{10292893-1B56-4F9A-A23A-27654775F02A}"/>
+    <workbookView xWindow="7050" yWindow="1875" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{10292893-1B56-4F9A-A23A-27654775F02A}"/>
   </bookViews>
   <sheets>
     <sheet name="NV" sheetId="9" r:id="rId1"/>
@@ -27,23 +27,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="15">
   <si>
     <t>Mã NV</t>
   </si>
@@ -58,15 +47,6 @@
   </si>
   <si>
     <t>KP.0002</t>
-  </si>
-  <si>
-    <t>KP.0003</t>
-  </si>
-  <si>
-    <t>KP.0004</t>
-  </si>
-  <si>
-    <t>KP.0005</t>
   </si>
   <si>
     <t>Ngày làm việc</t>
@@ -107,7 +87,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -521,14 +501,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15759177-BF27-4C7C-9ACB-C6E2150D6999}">
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -536,43 +516,11 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" t="s">
         <v>3</v>
       </c>
     </row>
@@ -584,24 +532,24 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22326FFD-AE1E-4653-957C-214778E20070}">
-  <dimension ref="A1:E35"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -611,10 +559,10 @@
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -624,10 +572,10 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -637,10 +585,10 @@
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -650,10 +598,10 @@
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -663,10 +611,10 @@
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -676,10 +624,10 @@
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -689,10 +637,10 @@
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -702,10 +650,10 @@
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -715,10 +663,10 @@
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -728,319 +676,7 @@
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
-        <v>2</v>
-      </c>
-      <c r="B12" s="1">
-        <v>46033</v>
-      </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" t="s">
-        <v>2</v>
-      </c>
-      <c r="B13" s="1">
-        <v>46034</v>
-      </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" t="s">
-        <v>2</v>
-      </c>
-      <c r="B14" s="1">
-        <v>46035</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B15" s="1">
-        <v>46036</v>
-      </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" t="s">
-        <v>2</v>
-      </c>
-      <c r="B16" s="1">
-        <v>46037</v>
-      </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" t="s">
-        <v>2</v>
-      </c>
-      <c r="B17" s="1">
-        <v>46038</v>
-      </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" t="s">
-        <v>2</v>
-      </c>
-      <c r="B18" s="1">
-        <v>46039</v>
-      </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" t="s">
-        <v>4</v>
-      </c>
-      <c r="B19" s="1">
-        <v>46023</v>
-      </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" t="s">
-        <v>4</v>
-      </c>
-      <c r="B20" s="1">
-        <v>46024</v>
-      </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" t="s">
-        <v>4</v>
-      </c>
-      <c r="B21" s="1">
-        <v>46025</v>
-      </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" t="s">
-        <v>4</v>
-      </c>
-      <c r="B22" s="1">
-        <v>46026</v>
-      </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" t="s">
-        <v>4</v>
-      </c>
-      <c r="B23" s="1">
-        <v>46027</v>
-      </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" t="s">
-        <v>4</v>
-      </c>
-      <c r="B24" s="1">
-        <v>46028</v>
-      </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" t="s">
-        <v>4</v>
-      </c>
-      <c r="B25" s="1">
-        <v>46029</v>
-      </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" t="s">
-        <v>4</v>
-      </c>
-      <c r="B26" s="1">
-        <v>46030</v>
-      </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" t="s">
-        <v>4</v>
-      </c>
-      <c r="B27" s="1">
-        <v>46031</v>
-      </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" t="s">
-        <v>4</v>
-      </c>
-      <c r="B28" s="1">
-        <v>46032</v>
-      </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="A29" t="s">
-        <v>4</v>
-      </c>
-      <c r="B29" s="1">
-        <v>46033</v>
-      </c>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" t="s">
-        <v>4</v>
-      </c>
-      <c r="B30" s="1">
-        <v>46034</v>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5">
-      <c r="A31" t="s">
-        <v>4</v>
-      </c>
-      <c r="B31" s="1">
-        <v>46035</v>
-      </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5">
-      <c r="A32" t="s">
-        <v>4</v>
-      </c>
-      <c r="B32" s="1">
-        <v>46036</v>
-      </c>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5">
-      <c r="A33" t="s">
-        <v>4</v>
-      </c>
-      <c r="B33" s="1">
-        <v>46037</v>
-      </c>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5">
-      <c r="A34" t="s">
-        <v>4</v>
-      </c>
-      <c r="B34" s="1">
-        <v>46038</v>
-      </c>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" t="s">
-        <v>4</v>
-      </c>
-      <c r="B35" s="1">
-        <v>46039</v>
-      </c>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1052,14 +688,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A66FBC5-37BD-4873-BDE4-B0CFF685044A}">
   <dimension ref="A1:AF4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="32" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B1">
         <v>1</v>
@@ -1155,7 +791,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:32">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1253,89 +889,90 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="3" spans="1:32">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="H3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="I3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="J3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="M3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="N3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="O3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="P3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="Q3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:32">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="H4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="I4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="J4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="M4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="N4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="O4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="P4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="Q4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor(robots): replace BuildChamCong robot with new implementation
Complete rewrite of the attendance tracking (Cham Cong) robot with improved structure.
Added new robot files (final.robot, original.robot) and updated type definitions
for Employee and InputConfig to support enhanced functionality. Binary Excel
files updated for input/output data processing.
</commit_message>
<xml_diff>
--- a/Library/Data/Input/Tạo dữ liệu tính lương.xlsx
+++ b/Library/Data/Input/Tạo dữ liệu tính lương.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29704"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huyhh1\workspace\kofax\cham-cong\Library\Data\Input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HoangTT\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B3A814C-F636-4F83-B75C-DDC998CF87D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{34B831DE-268F-417B-8CC5-72818CC02A58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8161C76B-DD29-4A17-8BC7-BEA913895D2B}"/>
   <bookViews>
-    <workbookView xWindow="7050" yWindow="1875" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{10292893-1B56-4F9A-A23A-27654775F02A}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{10292893-1B56-4F9A-A23A-27654775F02A}"/>
   </bookViews>
   <sheets>
     <sheet name="NV" sheetId="9" r:id="rId1"/>
@@ -27,12 +27,23 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="18">
   <si>
     <t>Mã NV</t>
   </si>
@@ -47,6 +58,15 @@
   </si>
   <si>
     <t>KP.0002</t>
+  </si>
+  <si>
+    <t>KP.0003</t>
+  </si>
+  <si>
+    <t>KP.0004</t>
+  </si>
+  <si>
+    <t>KP.0005</t>
   </si>
   <si>
     <t>Ngày làm việc</t>
@@ -87,7 +107,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -501,14 +521,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15759177-BF27-4C7C-9ACB-C6E2150D6999}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -516,11 +536,43 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
         <v>3</v>
       </c>
     </row>
@@ -532,24 +584,24 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22326FFD-AE1E-4653-957C-214778E20070}">
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -559,10 +611,10 @@
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -572,10 +624,10 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -585,10 +637,10 @@
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -598,10 +650,10 @@
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -611,10 +663,10 @@
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -624,10 +676,10 @@
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -637,10 +689,10 @@
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -650,10 +702,10 @@
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -663,10 +715,10 @@
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -676,7 +728,319 @@
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" t="s">
-        <v>8</v>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" s="1">
+        <v>46033</v>
+      </c>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" s="1">
+        <v>46034</v>
+      </c>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>2</v>
+      </c>
+      <c r="B14" s="1">
+        <v>46035</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" s="1">
+        <v>46036</v>
+      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16" s="1">
+        <v>46037</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>2</v>
+      </c>
+      <c r="B17" s="1">
+        <v>46038</v>
+      </c>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" s="1">
+        <v>46039</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" s="1">
+        <v>46023</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" s="1">
+        <v>46024</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" s="1">
+        <v>46025</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" s="1">
+        <v>46026</v>
+      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" s="1">
+        <v>46027</v>
+      </c>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" s="1">
+        <v>46028</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" s="1">
+        <v>46029</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" s="1">
+        <v>46030</v>
+      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" s="1">
+        <v>46031</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" s="1">
+        <v>46032</v>
+      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" s="1">
+        <v>46033</v>
+      </c>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" s="1">
+        <v>46034</v>
+      </c>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" s="1">
+        <v>46035</v>
+      </c>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" s="1">
+        <v>46036</v>
+      </c>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" s="1">
+        <v>46037</v>
+      </c>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" s="1">
+        <v>46038</v>
+      </c>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" t="s">
+        <v>4</v>
+      </c>
+      <c r="B35" s="1">
+        <v>46039</v>
+      </c>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -688,14 +1052,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A66FBC5-37BD-4873-BDE4-B0CFF685044A}">
   <dimension ref="A1:AF4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="32" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B1">
         <v>1</v>
@@ -791,7 +1155,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -889,90 +1253,89 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="I3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="J3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="M3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="N3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="O3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="P3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="Q3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="I4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="J4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="M4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="N4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="O4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="P4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="Q4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>